<commit_message>
Sync mensal motoristas: 4 atualizados, 3 novos
Atualizados:
- Ewerton de Paula Abreu: ZONAS_PREFERIDAS reordenado conforme resposta mais recente (10/08/2026)
- Carlos Eduardo de Souza: removido "VIAGENS" indevido de ZONAS_PREFERIDAS
- Renato Forte: ACEITA_VIAGENS SIM -> NAO (nao selecionou opcao de viagens na resposta)
- Gabriel Ferreira de Souza: removido "VIAGENS" indevido de ZONAS_PREFERIDAS

NOVOS (precisam de AGENT_ID_VUUPT preenchido manualmente):
- Ricardo Barbosa do Nascimento
- Marcio Dell Aringa
- Caio da Silva Bezerra
</commit_message>
<xml_diff>
--- a/dados/BD_MOTORISTAS.xlsx
+++ b/dados/BD_MOTORISTAS.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="20370" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Motoristas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Motoristas" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -760,7 +760,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>CENTRO,ZONA NORTE,ZONA SUL,ZONA OESTE</t>
+          <t>ZONA NORTE,CENTRO,ZONA OESTE,ZONA SUL</t>
         </is>
       </c>
     </row>
@@ -1057,7 +1057,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>ABCD,VIAGENS,ZONA LESTE,ZONA SUL</t>
+          <t>ABCD,ZONA LESTE,ZONA SUL</t>
         </is>
       </c>
     </row>
@@ -1072,7 +1072,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NAO</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1123,7 +1123,97 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>ZONA NORTE,ZONA OESTE,VIAGENS,OSASCO-BARUERI-ALPHAVILLE</t>
+          <t>ZONA NORTE,ZONA OESTE,OSASCO-BARUERI-ALPHAVILLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Ricardo Barbosa do Nascimento</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>COTIA-EMBU-TABOAO,OSASCO-BARUERI-ALPHAVILLE,ZONA OESTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Marcio Dell Aringa</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>ZONA LESTE,ABCD,ZONA NORTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Caio da Silva Bezerra</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>ZONA NORTE,ZONA OESTE,CENTRO,ZONA SUL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Preencher AGENT_ID_VUUPT de Ricardo Barbosa (47339) e Marcio Dell Aringa (31828) e ativar
Caio da Silva Bezerra segue ATIVO=NAO: ainda sem cadastro de agente no Vuupt.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/BD_MOTORISTAS.xlsx
+++ b/dados/BD_MOTORISTAS.xlsx
@@ -1128,6 +1128,9 @@
       </c>
     </row>
     <row r="22">
+      <c r="A22" t="n">
+        <v>47339</v>
+      </c>
       <c r="C22" t="inlineStr">
         <is>
           <t>Ricardo Barbosa do Nascimento</t>
@@ -1148,7 +1151,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>NAO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1158,6 +1161,9 @@
       </c>
     </row>
     <row r="23">
+      <c r="A23" t="n">
+        <v>31828</v>
+      </c>
       <c r="C23" t="inlineStr">
         <is>
           <t>Marcio Dell Aringa</t>
@@ -1178,7 +1184,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>NAO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">

</xml_diff>

<commit_message>
Cadastra motorista Jairo Domingues Abreu em BD_MOTORISTAS.xlsx
agent_id 46418, ativo, não aceita viagens em lote, zonas Guarulhos/
Zona Norte/Centro/Zona Leste, placa PXW0C92.
</commit_message>
<xml_diff>
--- a/dados/BD_MOTORISTAS.xlsx
+++ b/dados/BD_MOTORISTAS.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1433,15 +1433,62 @@
           <t>ZONA NORTE,ZONA OESTE,GUARULHOS</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>11984344347</t>
-        </is>
+      <c r="I25" t="n">
+        <v>11984344347</v>
       </c>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
           <t>FUP1D50</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>46418</v>
+      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Jairo Domingues Abreu</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>GUARULHOS,ZONA NORTE,CENTRO,ZONA LESTE</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>+5511922305832</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>JairoAbreu@Freshlog.com</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>PXW0C92</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Desliga notificacoes automaticas externas e adiciona botao de ocorrencia na Fila de Acao
Notificacoes automaticas de e-mail pra embarcador/transportadora (dia fixo,
agendamento pendente, transportadoras, pedidos em espera, ocorrencia de
insucesso) agora sao controladas por config.yaml: notificacoes_automaticas.ativo.
A ocorrencia de insucesso ganha um botao "Notificar" na Fila de Acao da Torre
de Controle, mesmo padrao do "Duplicar pedido" ja existente, pra disparo
manual item a item.

Tambem inclui trabalho em andamento em paralelo: reforma da regua de KPIs da
Torre (dia/semana/mes/trimestre, atual x anterior), progresso/ETA ao vivo dos
agentes rodando, e o fluxo de notificar cliente pra retirada em pedidos parados.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/BD_MOTORISTAS.xlsx
+++ b/dados/BD_MOTORISTAS.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -666,7 +666,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>09474142742</t>
+          <t>9474142742</t>
         </is>
       </c>
     </row>
@@ -1670,6 +1670,104 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>50190</v>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Samuel Fugazza Neto</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>ZONA NORTE,ZONA OESTE,ZONA SUL,ZONA LESTE</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>5511940851740</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>sn@freshlog.com.br</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>42993322885</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>50191</v>
+      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Iago Mendes</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>ZONA NORTE,ZONA OESTE,ZONA SUL,ZONA LESTE</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>5511970239954</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>im@freshlog.com.br</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>42640649884</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cadastra motorista Rafael Batista Ribeiro no BD_MOTORISTAS
Agent VUUPT 50199, Seg-Sex, VAN/HR, sem restricao de zona.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/BD_MOTORISTAS.xlsx
+++ b/dados/BD_MOTORISTAS.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,68 +413,73 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:M30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>AGENT_ID_VUUPT</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>VEHICLE_ID_VUUPT</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>NOME_MOTORISTA</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>ACEITA_VIAGENS</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>DIAS_DISPONIVEIS</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>MAX_ROTAS_DIA</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>ATIVO</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>ZONAS_PREFERIDAS</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>TELEFONE_MOTORISTA</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>EMAIL_MOTORISTA</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>PLACA</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>CPF_MOTORISTA</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>TIPO_VEICULO</t>
         </is>
       </c>
     </row>
@@ -535,6 +528,7 @@
           <t>13415403831</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -577,6 +571,7 @@
           <t>40424591880</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -623,6 +618,7 @@
           <t>34822303829</t>
         </is>
       </c>
+      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -669,6 +665,7 @@
           <t>9474142742</t>
         </is>
       </c>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -715,6 +712,7 @@
           <t>43877896898</t>
         </is>
       </c>
+      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -761,6 +759,7 @@
           <t>28090589898</t>
         </is>
       </c>
+      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -807,6 +806,7 @@
           <t>47944413800</t>
         </is>
       </c>
+      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -853,6 +853,7 @@
           <t>30700585826</t>
         </is>
       </c>
+      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -899,6 +900,7 @@
           <t>22425592814</t>
         </is>
       </c>
+      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -945,6 +947,7 @@
           <t>38938114864</t>
         </is>
       </c>
+      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -991,6 +994,7 @@
           <t>28209297880</t>
         </is>
       </c>
+      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1037,6 +1041,7 @@
           <t>37026112821</t>
         </is>
       </c>
+      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1083,6 +1088,7 @@
           <t>44578842860</t>
         </is>
       </c>
+      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1125,6 +1131,7 @@
           <t>46119496807</t>
         </is>
       </c>
+      <c r="M15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1163,6 +1170,7 @@
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1209,6 +1217,7 @@
           <t>34944268807</t>
         </is>
       </c>
+      <c r="M17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1251,6 +1260,7 @@
           <t>43125943841</t>
         </is>
       </c>
+      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1297,6 +1307,7 @@
           <t>19277023805</t>
         </is>
       </c>
+      <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1343,6 +1354,7 @@
           <t>11496700880</t>
         </is>
       </c>
+      <c r="M20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1389,6 +1401,7 @@
           <t>46065478806</t>
         </is>
       </c>
+      <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1435,6 +1448,7 @@
           <t>31064536808</t>
         </is>
       </c>
+      <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1481,6 +1495,7 @@
           <t>27466740847</t>
         </is>
       </c>
+      <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1527,6 +1542,7 @@
           <t>47944413800</t>
         </is>
       </c>
+      <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1575,6 +1591,7 @@
           <t>22618919890</t>
         </is>
       </c>
+      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1627,6 +1644,7 @@
           <t>41073933806</t>
         </is>
       </c>
+      <c r="M26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1669,6 +1687,7 @@
           <t>11111111111</t>
         </is>
       </c>
+      <c r="M27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1717,6 +1736,7 @@
           <t>42993322885</t>
         </is>
       </c>
+      <c r="M28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1751,10 +1771,8 @@
           <t>ZONA NORTE,ZONA OESTE,ZONA SUL,ZONA LESTE</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>5511970239954</t>
-        </is>
+      <c r="I29" t="n">
+        <v>5511970239954</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
@@ -1765,6 +1783,54 @@
       <c r="L29" t="inlineStr">
         <is>
           <t>42640649884</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>50199</v>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Rafael Batista Ribeiro</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>11995109716</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>EMU6742</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>VAN_HR</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Lalamove: motorista virtual no planejamento cria pedido, carimba codigo no titulo Vuupt e sync conclui servicos
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/BD_MOTORISTAS.xlsx
+++ b/dados/BD_MOTORISTAS.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M30"/>
+  <dimension ref="A1:M31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -487,7 +487,6 @@
       <c r="A2" t="n">
         <v>33821</v>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>Adriano Alves</t>
@@ -516,8 +515,6 @@
           <t>ZONA NORTE,GUARULHOS,ZONA LESTE</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
           <t>PZD7G26</t>
@@ -528,13 +525,11 @@
           <t>13415403831</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
         <v>46415</v>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>Bruno Espinoza Russo</t>
@@ -563,21 +558,16 @@
           <t>ZONA NORTE,ZONA OESTE,OSASCO-BARUERI-ALPHAVILLE,COTIA-EMBU-TABOAO</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>40424591880</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
         <v>45594</v>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>Cicero Barbosa da silva</t>
@@ -606,8 +596,6 @@
           <t>ZONA NORTE</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
           <t>OQH7B64</t>
@@ -618,13 +606,11 @@
           <t>34822303829</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
         <v>42642</v>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>Clayson martins Pereira</t>
@@ -653,8 +639,6 @@
           <t>ZONA NORTE,ABCD,COTIA-EMBU-TABOAO</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
           <t>EZD9B14</t>
@@ -665,13 +649,11 @@
           <t>9474142742</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
         <v>44935</v>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>Diego Nascimento da Silva</t>
@@ -700,8 +682,6 @@
           <t>OSASCO-BARUERI-ALPHAVILLE,ABCD,ZONA OESTE</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
           <t xml:space="preserve">RVD4D10 </t>
@@ -712,13 +692,11 @@
           <t>43877896898</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
         <v>29252</v>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>Edvaldo De Jesus Santos Junior</t>
@@ -747,8 +725,6 @@
           <t>OSASCO-BARUERI-ALPHAVILLE,ABCD,GUARULHOS</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>FAW8I34</t>
@@ -759,13 +735,11 @@
           <t>28090589898</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
         <v>47424</v>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>Erick Gomes Oliveira</t>
@@ -794,8 +768,6 @@
           <t>ZONA NORTE,ZONA OESTE,CENTRO</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>EDY1E57</t>
@@ -806,13 +778,11 @@
           <t>47944413800</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
         <v>45149</v>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>Erivan soares de oliveira</t>
@@ -841,8 +811,6 @@
           <t>GUARULHOS,ZONA NORTE,ZONA LESTE,ABCD</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>FYD1E68</t>
@@ -853,13 +821,11 @@
           <t>30700585826</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
         <v>29253</v>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>Ewerton de Paula Abreu</t>
@@ -888,8 +854,6 @@
           <t>ZONA NORTE,CENTRO,ZONA OESTE,ZONA SUL</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
           <t>EAA0985</t>
@@ -900,13 +864,11 @@
           <t>22425592814</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
         <v>45422</v>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>Fagner Macedo</t>
@@ -935,8 +897,6 @@
           <t>ZONA OESTE,ZONA NORTE,CENTRO</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
           <t>FQJ7F16</t>
@@ -947,13 +907,11 @@
           <t>38938114864</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
         <v>47083</v>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>Fábio Barbosa</t>
@@ -982,8 +940,6 @@
           <t>ZONA LESTE,GUARULHOS,ABCD</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
           <t xml:space="preserve">PWI9H55 </t>
@@ -994,13 +950,11 @@
           <t>28209297880</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
         <v>47039</v>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>Hedgar Miralha Nascimento</t>
@@ -1029,8 +983,6 @@
           <t>ZONA NORTE,ZONA OESTE,ZONA LESTE,GUARULHOS</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
           <t>EFW3059</t>
@@ -1041,13 +993,11 @@
           <t>37026112821</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
         <v>35339</v>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>João Victor Galdino Gonçalves</t>
@@ -1076,8 +1026,6 @@
           <t>OSASCO-BARUERI-ALPHAVILLE,ZONA NORTE,COTIA-EMBU-TABOAO</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
           <t>FVE0I20</t>
@@ -1088,13 +1036,11 @@
           <t>44578842860</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
         <v>45795</v>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>Renato Rodzewics Silva</t>
@@ -1123,21 +1069,16 @@
           <t>ZONA NORTE,ABCD,OSASCO-BARUERI-ALPHAVILLE</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
           <t>46119496807</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
         <v>46454</v>
       </c>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
           <t>Caio da Silva Bezerra (Erick 2)</t>
@@ -1166,17 +1107,11 @@
           <t>ZONA NORTE,ZONA OESTE,CENTRO</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
         <v>47084</v>
       </c>
-      <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
           <t>Vinícius Oliveira Correia</t>
@@ -1205,8 +1140,6 @@
           <t>ZONA NORTE,ZONA OESTE,ZONA LESTE</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
           <t>RUV9D51</t>
@@ -1217,13 +1150,11 @@
           <t>34944268807</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
         <v>46474</v>
       </c>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
           <t>Ériclis Castro Nunes</t>
@@ -1252,21 +1183,16 @@
           <t>CENTRO,ZONA OESTE,GUARULHOS</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
           <t>43125943841</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
         <v>48547</v>
       </c>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
           <t>Carlos Eduardo de Souza</t>
@@ -1295,8 +1221,6 @@
           <t>ABCD,ZONA LESTE,ZONA SUL</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
           <t>GGO8B38</t>
@@ -1307,13 +1231,11 @@
           <t>19277023805</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
         <v>48907</v>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
           <t>Renato Forte</t>
@@ -1342,8 +1264,6 @@
           <t>ZONA NORTE,CENTRO,ZONA LESTE,GUARULHOS</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
           <t>ATW2C46</t>
@@ -1354,13 +1274,11 @@
           <t>11496700880</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
         <v>48546</v>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
           <t>Gabriel Ferreira de Souza</t>
@@ -1389,8 +1307,6 @@
           <t>ZONA NORTE,ZONA OESTE,OSASCO-BARUERI-ALPHAVILLE</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
           <t>RTJ7E66</t>
@@ -1401,13 +1317,11 @@
           <t>46065478806</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
         <v>47339</v>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
           <t>Ricardo Barbosa do Nascimento</t>
@@ -1436,8 +1350,6 @@
           <t>COTIA-EMBU-TABOAO,OSASCO-BARUERI-ALPHAVILLE,ZONA OESTE</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
           <t>PUX6D34</t>
@@ -1448,13 +1360,11 @@
           <t>31064536808</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
         <v>31828</v>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
           <t>Marcio Dell Aringa</t>
@@ -1483,8 +1393,6 @@
           <t>ZONA LESTE,ABCD,ZONA NORTE</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
           <t>NYA4J21</t>
@@ -1495,13 +1403,11 @@
           <t>27466740847</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
         <v>47424</v>
       </c>
-      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
           <t>Erick Gomes Oliveira - CARRO 2</t>
@@ -1530,8 +1436,6 @@
           <t>ZONA NORTE,ZONA OESTE,CENTRO</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
         <is>
           <t>FVK3G29</t>
@@ -1542,13 +1446,11 @@
           <t>47944413800</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
         <v>50016</v>
       </c>
-      <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
           <t>Wellington Bittencourt dos Santos</t>
@@ -1580,7 +1482,6 @@
       <c r="I25" t="n">
         <v>11984344347</v>
       </c>
-      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
           <t>FUP1D50</t>
@@ -1591,13 +1492,11 @@
           <t>22618919890</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
         <v>46418</v>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
           <t>Jairo Domingues Abreu</t>
@@ -1644,13 +1543,11 @@
           <t>41073933806</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
         <v>28438</v>
       </c>
-      <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
           <t>Hugo Maçol Sousa (TESTE)</t>
@@ -1679,21 +1576,16 @@
           <t>ZONA NORTE,ZONA SUL,ZONA LESTE,ZONA OESTE,CENTRO,GUARULHOS,ABCD,OSASCO - BARUERI - SANTANA DE PARNAÍBA - ALPHAVILLE,COTIA - EMBU DAS ARTES - TABOÃO</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
           <t>11111111111</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
         <v>50190</v>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
           <t>Samuel Fugazza Neto</t>
@@ -1730,19 +1622,16 @@
           <t>sn@freshlog.com.br</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
           <t>42993322885</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
         <v>50191</v>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
           <t>Iago Mendes</t>
@@ -1779,19 +1668,16 @@
           <t>im@freshlog.com.br</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
           <t>42640649884</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
         <v>50199</v>
       </c>
-      <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
           <t>Rafael Batista Ribeiro</t>
@@ -1815,22 +1701,42 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
           <t>11995109716</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
           <t>EMU6742</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr">
         <is>
           <t>VAN_HR</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>50258</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>LALAMOVE (virtual)</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>99</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>SIM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Motoristas: vincula carros aos agentes no Vuupt e preenche VEHICLE_ID_VUUPT
vincular_veiculos_motoristas.py cruza a PLACA da planilha com GET /vehicles
e, com match unico, faz PUT /users/{agent_id} vehicle_id (parcial, testado
no agente TESTE) e preenche a coluna VEHICLE_ID_VUUPT da linha. Com a
coluna preenchida, criar_rotas_diarias/rascunhos_rota passam a mandar o
vehicle_id no POST /routes -- rota nasce com o carro no Vuupt.

Rodado em producao 01/09: 19 vinculos novos + 2 ja existentes, 22 linhas
preenchidas; 8 linhas sem placa ficam de fora (avisadas no log).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/BD_MOTORISTAS.xlsx
+++ b/dados/BD_MOTORISTAS.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,67 +429,67 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>AGENT_ID_VUUPT</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>VEHICLE_ID_VUUPT</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>NOME_MOTORISTA</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>ACEITA_VIAGENS</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>DIAS_DISPONIVEIS</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>MAX_ROTAS_DIA</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>ATIVO</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>ZONAS_PREFERIDAS</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>TELEFONE_MOTORISTA</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>EMAIL_MOTORISTA</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>PLACA</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>CPF_MOTORISTA</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>TIPO_VEICULO</t>
         </is>
@@ -487,6 +499,9 @@
       <c r="A2" t="n">
         <v>33821</v>
       </c>
+      <c r="B2" t="n">
+        <v>37259</v>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>Adriano Alves</t>
@@ -515,21 +530,23 @@
           <t>ZONA NORTE,GUARULHOS,ZONA LESTE</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
           <t>PZD7G26</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>13415403831</t>
-        </is>
-      </c>
+      <c r="L2" t="n">
+        <v>13415403831</v>
+      </c>
+      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
         <v>46415</v>
       </c>
+      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>Bruno Espinoza Russo</t>
@@ -558,16 +575,21 @@
           <t>ZONA NORTE,ZONA OESTE,OSASCO-BARUERI-ALPHAVILLE,COTIA-EMBU-TABOAO</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>40424591880</t>
-        </is>
-      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="n">
+        <v>40424591880</v>
+      </c>
+      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
         <v>45594</v>
       </c>
+      <c r="B4" t="n">
+        <v>96978</v>
+      </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>Cicero Barbosa da silva</t>
@@ -596,21 +618,25 @@
           <t>ZONA NORTE</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
           <t>OQH7B64</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>34822303829</t>
-        </is>
-      </c>
+      <c r="L4" t="n">
+        <v>34822303829</v>
+      </c>
+      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
         <v>42642</v>
       </c>
+      <c r="B5" t="n">
+        <v>87595</v>
+      </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>Clayson martins Pereira</t>
@@ -639,21 +665,25 @@
           <t>ZONA NORTE,ABCD,COTIA-EMBU-TABOAO</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
           <t>EZD9B14</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>9474142742</t>
-        </is>
-      </c>
+      <c r="L5" t="n">
+        <v>9474142742</v>
+      </c>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
         <v>44935</v>
       </c>
+      <c r="B6" t="n">
+        <v>96064</v>
+      </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>Diego Nascimento da Silva</t>
@@ -682,21 +712,25 @@
           <t>OSASCO-BARUERI-ALPHAVILLE,ABCD,ZONA OESTE</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
           <t xml:space="preserve">RVD4D10 </t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>43877896898</t>
-        </is>
-      </c>
+      <c r="L6" t="n">
+        <v>43877896898</v>
+      </c>
+      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
         <v>29252</v>
       </c>
+      <c r="B7" t="n">
+        <v>20758</v>
+      </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>Edvaldo De Jesus Santos Junior</t>
@@ -725,21 +759,25 @@
           <t>OSASCO-BARUERI-ALPHAVILLE,ABCD,GUARULHOS</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>FAW8I34</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>28090589898</t>
-        </is>
-      </c>
+      <c r="L7" t="n">
+        <v>28090589898</v>
+      </c>
+      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
         <v>47424</v>
       </c>
+      <c r="B8" t="n">
+        <v>102635</v>
+      </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>Erick Gomes Oliveira</t>
@@ -768,21 +806,25 @@
           <t>ZONA NORTE,ZONA OESTE,CENTRO</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>EDY1E57</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>47944413800</t>
-        </is>
-      </c>
+      <c r="L8" t="n">
+        <v>47944413800</v>
+      </c>
+      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
         <v>45149</v>
       </c>
+      <c r="B9" t="n">
+        <v>96167</v>
+      </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>Erivan soares de oliveira</t>
@@ -811,21 +853,25 @@
           <t>GUARULHOS,ZONA NORTE,ZONA LESTE,ABCD</t>
         </is>
       </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>FYD1E68</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>30700585826</t>
-        </is>
-      </c>
+      <c r="L9" t="n">
+        <v>30700585826</v>
+      </c>
+      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
         <v>29253</v>
       </c>
+      <c r="B10" t="n">
+        <v>20757</v>
+      </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>Ewerton de Paula Abreu</t>
@@ -854,21 +900,25 @@
           <t>ZONA NORTE,CENTRO,ZONA OESTE,ZONA SUL</t>
         </is>
       </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
           <t>EAA0985</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>22425592814</t>
-        </is>
-      </c>
+      <c r="L10" t="n">
+        <v>22425592814</v>
+      </c>
+      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
         <v>45422</v>
       </c>
+      <c r="B11" t="n">
+        <v>96671</v>
+      </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>Fagner Macedo</t>
@@ -897,21 +947,25 @@
           <t>ZONA OESTE,ZONA NORTE,CENTRO</t>
         </is>
       </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
           <t>FQJ7F16</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>38938114864</t>
-        </is>
-      </c>
+      <c r="L11" t="n">
+        <v>38938114864</v>
+      </c>
+      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
         <v>47083</v>
       </c>
+      <c r="B12" t="n">
+        <v>103183</v>
+      </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>Fábio Barbosa</t>
@@ -940,21 +994,25 @@
           <t>ZONA LESTE,GUARULHOS,ABCD</t>
         </is>
       </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
           <t xml:space="preserve">PWI9H55 </t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>28209297880</t>
-        </is>
-      </c>
+      <c r="L12" t="n">
+        <v>28209297880</v>
+      </c>
+      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
         <v>47039</v>
       </c>
+      <c r="B13" t="n">
+        <v>103160</v>
+      </c>
       <c r="C13" t="inlineStr">
         <is>
           <t>Hedgar Miralha Nascimento</t>
@@ -983,21 +1041,25 @@
           <t>ZONA NORTE,ZONA OESTE,ZONA LESTE,GUARULHOS</t>
         </is>
       </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
           <t>EFW3059</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>37026112821</t>
-        </is>
-      </c>
+      <c r="L13" t="n">
+        <v>37026112821</v>
+      </c>
+      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
         <v>35339</v>
       </c>
+      <c r="B14" t="n">
+        <v>52356</v>
+      </c>
       <c r="C14" t="inlineStr">
         <is>
           <t>João Victor Galdino Gonçalves</t>
@@ -1026,21 +1088,23 @@
           <t>OSASCO-BARUERI-ALPHAVILLE,ZONA NORTE,COTIA-EMBU-TABOAO</t>
         </is>
       </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
           <t>FVE0I20</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>44578842860</t>
-        </is>
-      </c>
+      <c r="L14" t="n">
+        <v>44578842860</v>
+      </c>
+      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
         <v>45795</v>
       </c>
+      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>Renato Rodzewics Silva</t>
@@ -1069,16 +1133,19 @@
           <t>ZONA NORTE,ABCD,OSASCO-BARUERI-ALPHAVILLE</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>46119496807</t>
-        </is>
-      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="n">
+        <v>46119496807</v>
+      </c>
+      <c r="M15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
         <v>46454</v>
       </c>
+      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
           <t>Caio da Silva Bezerra (Erick 2)</t>
@@ -1107,11 +1174,19 @@
           <t>ZONA NORTE,ZONA OESTE,CENTRO</t>
         </is>
       </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
         <v>47084</v>
       </c>
+      <c r="B17" t="n">
+        <v>103182</v>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
           <t>Vinícius Oliveira Correia</t>
@@ -1140,21 +1215,23 @@
           <t>ZONA NORTE,ZONA OESTE,ZONA LESTE</t>
         </is>
       </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
           <t>RUV9D51</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>34944268807</t>
-        </is>
-      </c>
+      <c r="L17" t="n">
+        <v>34944268807</v>
+      </c>
+      <c r="M17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
         <v>46474</v>
       </c>
+      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
           <t>Ériclis Castro Nunes</t>
@@ -1183,16 +1260,21 @@
           <t>CENTRO,ZONA OESTE,GUARULHOS</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>43125943841</t>
-        </is>
-      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="n">
+        <v>43125943841</v>
+      </c>
+      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
         <v>48547</v>
       </c>
+      <c r="B19" t="n">
+        <v>104257</v>
+      </c>
       <c r="C19" t="inlineStr">
         <is>
           <t>Carlos Eduardo de Souza</t>
@@ -1221,21 +1303,25 @@
           <t>ABCD,ZONA LESTE,ZONA SUL</t>
         </is>
       </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
           <t>GGO8B38</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>19277023805</t>
-        </is>
-      </c>
+      <c r="L19" t="n">
+        <v>19277023805</v>
+      </c>
+      <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
         <v>48907</v>
       </c>
+      <c r="B20" t="n">
+        <v>104506</v>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
           <t>Renato Forte</t>
@@ -1264,21 +1350,25 @@
           <t>ZONA NORTE,CENTRO,ZONA LESTE,GUARULHOS</t>
         </is>
       </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
           <t>ATW2C46</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>11496700880</t>
-        </is>
-      </c>
+      <c r="L20" t="n">
+        <v>11496700880</v>
+      </c>
+      <c r="M20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
         <v>48546</v>
       </c>
+      <c r="B21" t="n">
+        <v>104256</v>
+      </c>
       <c r="C21" t="inlineStr">
         <is>
           <t>Gabriel Ferreira de Souza</t>
@@ -1307,21 +1397,25 @@
           <t>ZONA NORTE,ZONA OESTE,OSASCO-BARUERI-ALPHAVILLE</t>
         </is>
       </c>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
           <t>RTJ7E66</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>46065478806</t>
-        </is>
-      </c>
+      <c r="L21" t="n">
+        <v>46065478806</v>
+      </c>
+      <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
         <v>47339</v>
       </c>
+      <c r="B22" t="n">
+        <v>103339</v>
+      </c>
       <c r="C22" t="inlineStr">
         <is>
           <t>Ricardo Barbosa do Nascimento</t>
@@ -1350,21 +1444,25 @@
           <t>COTIA-EMBU-TABOAO,OSASCO-BARUERI-ALPHAVILLE,ZONA OESTE</t>
         </is>
       </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
           <t>PUX6D34</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>31064536808</t>
-        </is>
-      </c>
+      <c r="L22" t="n">
+        <v>31064536808</v>
+      </c>
+      <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
         <v>31828</v>
       </c>
+      <c r="B23" t="n">
+        <v>22570</v>
+      </c>
       <c r="C23" t="inlineStr">
         <is>
           <t>Marcio Dell Aringa</t>
@@ -1393,21 +1491,25 @@
           <t>ZONA LESTE,ABCD,ZONA NORTE</t>
         </is>
       </c>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
           <t>NYA4J21</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>27466740847</t>
-        </is>
-      </c>
+      <c r="L23" t="n">
+        <v>27466740847</v>
+      </c>
+      <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
         <v>47424</v>
       </c>
+      <c r="B24" t="n">
+        <v>103406</v>
+      </c>
       <c r="C24" t="inlineStr">
         <is>
           <t>Erick Gomes Oliveira - CARRO 2</t>
@@ -1436,21 +1538,25 @@
           <t>ZONA NORTE,ZONA OESTE,CENTRO</t>
         </is>
       </c>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
         <is>
           <t>FVK3G29</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>47944413800</t>
-        </is>
-      </c>
+      <c r="L24" t="n">
+        <v>47944413800</v>
+      </c>
+      <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
         <v>50016</v>
       </c>
+      <c r="B25" t="n">
+        <v>106040</v>
+      </c>
       <c r="C25" t="inlineStr">
         <is>
           <t>Wellington Bittencourt dos Santos</t>
@@ -1482,21 +1588,24 @@
       <c r="I25" t="n">
         <v>11984344347</v>
       </c>
+      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
           <t>FUP1D50</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>22618919890</t>
-        </is>
-      </c>
+      <c r="L25" t="n">
+        <v>22618919890</v>
+      </c>
+      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
         <v>46418</v>
       </c>
+      <c r="B26" t="n">
+        <v>102703</v>
+      </c>
       <c r="C26" t="inlineStr">
         <is>
           <t>Jairo Domingues Abreu</t>
@@ -1538,16 +1647,16 @@
           <t>PXW0C92</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>41073933806</t>
-        </is>
-      </c>
+      <c r="L26" t="n">
+        <v>41073933806</v>
+      </c>
+      <c r="M26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
         <v>28438</v>
       </c>
+      <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
           <t>Hugo Maçol Sousa (TESTE)</t>
@@ -1576,16 +1685,19 @@
           <t>ZONA NORTE,ZONA SUL,ZONA LESTE,ZONA OESTE,CENTRO,GUARULHOS,ABCD,OSASCO - BARUERI - SANTANA DE PARNAÍBA - ALPHAVILLE,COTIA - EMBU DAS ARTES - TABOÃO</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>11111111111</t>
-        </is>
-      </c>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="n">
+        <v>11111111111</v>
+      </c>
+      <c r="M27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
         <v>50190</v>
       </c>
+      <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
           <t>Samuel Fugazza Neto</t>
@@ -1622,16 +1734,17 @@
           <t>sn@freshlog.com.br</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>42993322885</t>
-        </is>
-      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="n">
+        <v>42993322885</v>
+      </c>
+      <c r="M28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
         <v>50191</v>
       </c>
+      <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
           <t>Iago Mendes</t>
@@ -1668,16 +1781,19 @@
           <t>im@freshlog.com.br</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>42640649884</t>
-        </is>
-      </c>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="n">
+        <v>42640649884</v>
+      </c>
+      <c r="M29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
         <v>50199</v>
       </c>
+      <c r="B30" t="n">
+        <v>106175</v>
+      </c>
       <c r="C30" t="inlineStr">
         <is>
           <t>Rafael Batista Ribeiro</t>
@@ -1701,16 +1817,17 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>11995109716</t>
-        </is>
-      </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="n">
+        <v>11995109716</v>
+      </c>
+      <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
           <t>EMU6742</t>
         </is>
       </c>
+      <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr">
         <is>
           <t>VAN_HR</t>
@@ -1721,6 +1838,7 @@
       <c r="A31" t="n">
         <v>50258</v>
       </c>
+      <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
           <t>LALAMOVE (virtual)</t>
@@ -1731,6 +1849,7 @@
           <t>NAO</t>
         </is>
       </c>
+      <c r="E31" t="inlineStr"/>
       <c r="F31" t="n">
         <v>99</v>
       </c>
@@ -1739,6 +1858,12 @@
           <t>SIM</t>
         </is>
       </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
BD_Motoristas: remove Diego Nascimento, Carlos Eduardo, Bruno e Ériclis da lista
Pedido do Hugo (10/09). Linhas apagadas da planilha (agent_ids 44935,
48547, 46415, 46474); nenhum deles tinha login no núcleo.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/BD_MOTORISTAS.xlsx
+++ b/dados/BD_MOTORISTAS.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M31"/>
+  <dimension ref="A1:M27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -537,19 +537,23 @@
           <t>PZD7G26</t>
         </is>
       </c>
-      <c r="L2" t="n">
-        <v>13415403831</v>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>13415403831</t>
+        </is>
       </c>
       <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>46415</v>
-      </c>
-      <c r="B3" t="inlineStr"/>
+        <v>45594</v>
+      </c>
+      <c r="B3" t="n">
+        <v>96978</v>
+      </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Bruno Espinoza Russo</t>
+          <t>Cicero Barbosa da silva</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -567,37 +571,43 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>NAO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>ZONA NORTE,ZONA OESTE,OSASCO-BARUERI-ALPHAVILLE,COTIA-EMBU-TABOAO</t>
+          <t>ZONA NORTE</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="n">
-        <v>40424591880</v>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>OQH7B64</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>34822303829</t>
+        </is>
       </c>
       <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>45594</v>
+        <v>42642</v>
       </c>
       <c r="B4" t="n">
-        <v>96978</v>
+        <v>87595</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Cicero Barbosa da silva</t>
+          <t>Clayson martins Pereira</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>NAO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -615,31 +625,33 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>ZONA NORTE</t>
+          <t>ZONA NORTE,ABCD,COTIA-EMBU-TABOAO</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>OQH7B64</t>
-        </is>
-      </c>
-      <c r="L4" t="n">
-        <v>34822303829</v>
+          <t>EZD9B14</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>9474142742</t>
+        </is>
       </c>
       <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>42642</v>
+        <v>29252</v>
       </c>
       <c r="B5" t="n">
-        <v>87595</v>
+        <v>20758</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Clayson martins Pereira</t>
+          <t>Edvaldo De Jesus Santos Junior</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -657,41 +669,43 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NAO</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>ZONA NORTE,ABCD,COTIA-EMBU-TABOAO</t>
+          <t>OSASCO-BARUERI-ALPHAVILLE,ABCD,GUARULHOS</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>EZD9B14</t>
-        </is>
-      </c>
-      <c r="L5" t="n">
-        <v>9474142742</v>
+          <t>FAW8I34</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>28090589898</t>
+        </is>
       </c>
       <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>44935</v>
+        <v>47424</v>
       </c>
       <c r="B6" t="n">
-        <v>96064</v>
+        <v>102635</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Diego Nascimento da Silva</t>
+          <t>Erick Gomes Oliveira</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NAO</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -709,36 +723,38 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>OSASCO-BARUERI-ALPHAVILLE,ABCD,ZONA OESTE</t>
+          <t>ZONA NORTE,ZONA OESTE,CENTRO</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t xml:space="preserve">RVD4D10 </t>
-        </is>
-      </c>
-      <c r="L6" t="n">
-        <v>43877896898</v>
+          <t>EDY1E57</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>47944413800</t>
+        </is>
       </c>
       <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>29252</v>
+        <v>45149</v>
       </c>
       <c r="B7" t="n">
-        <v>20758</v>
+        <v>96167</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Edvaldo De Jesus Santos Junior</t>
+          <t>Erivan soares de oliveira</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NAO</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -751,36 +767,38 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>NAO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>OSASCO-BARUERI-ALPHAVILLE,ABCD,GUARULHOS</t>
+          <t>GUARULHOS,ZONA NORTE,ZONA LESTE,ABCD</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>FAW8I34</t>
-        </is>
-      </c>
-      <c r="L7" t="n">
-        <v>28090589898</v>
+          <t>FYD1E68</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>30700585826</t>
+        </is>
       </c>
       <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>47424</v>
+        <v>29253</v>
       </c>
       <c r="B8" t="n">
-        <v>102635</v>
+        <v>20757</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Erick Gomes Oliveira</t>
+          <t>Ewerton de Paula Abreu</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -803,36 +821,38 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>ZONA NORTE,ZONA OESTE,CENTRO</t>
+          <t>ZONA NORTE,CENTRO,ZONA OESTE,ZONA SUL</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>EDY1E57</t>
-        </is>
-      </c>
-      <c r="L8" t="n">
-        <v>47944413800</v>
+          <t>EAA0985</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>22425592814</t>
+        </is>
       </c>
       <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>45149</v>
+        <v>45422</v>
       </c>
       <c r="B9" t="n">
-        <v>96167</v>
+        <v>96671</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Erivan soares de oliveira</t>
+          <t>Fagner Macedo</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>NAO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -850,36 +870,38 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>GUARULHOS,ZONA NORTE,ZONA LESTE,ABCD</t>
+          <t>ZONA OESTE,ZONA NORTE,CENTRO</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>FYD1E68</t>
-        </is>
-      </c>
-      <c r="L9" t="n">
-        <v>30700585826</v>
+          <t>FQJ7F16</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>38938114864</t>
+        </is>
       </c>
       <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>29253</v>
+        <v>47083</v>
       </c>
       <c r="B10" t="n">
-        <v>20757</v>
+        <v>103183</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Ewerton de Paula Abreu</t>
+          <t>Fábio Barbosa</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>NAO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -897,36 +919,38 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>ZONA NORTE,CENTRO,ZONA OESTE,ZONA SUL</t>
+          <t>ZONA LESTE,GUARULHOS,ABCD</t>
         </is>
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>EAA0985</t>
-        </is>
-      </c>
-      <c r="L10" t="n">
-        <v>22425592814</v>
+          <t xml:space="preserve">PWI9H55 </t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>28209297880</t>
+        </is>
       </c>
       <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>45422</v>
+        <v>47039</v>
       </c>
       <c r="B11" t="n">
-        <v>96671</v>
+        <v>103160</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fagner Macedo</t>
+          <t>Hedgar Miralha Nascimento</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NAO</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -944,31 +968,33 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>ZONA OESTE,ZONA NORTE,CENTRO</t>
+          <t>ZONA NORTE,ZONA OESTE,ZONA LESTE,GUARULHOS</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
-          <t>FQJ7F16</t>
-        </is>
-      </c>
-      <c r="L11" t="n">
-        <v>38938114864</v>
+          <t>EFW3059</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>37026112821</t>
+        </is>
       </c>
       <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>47083</v>
+        <v>35339</v>
       </c>
       <c r="B12" t="n">
-        <v>103183</v>
+        <v>52356</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Fábio Barbosa</t>
+          <t>João Victor Galdino Gonçalves</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -986,88 +1012,84 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NAO</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>ZONA LESTE,GUARULHOS,ABCD</t>
+          <t>OSASCO-BARUERI-ALPHAVILLE,ZONA NORTE,COTIA-EMBU-TABOAO</t>
         </is>
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t xml:space="preserve">PWI9H55 </t>
-        </is>
-      </c>
-      <c r="L12" t="n">
-        <v>28209297880</v>
+          <t>FVE0I20</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>44578842860</t>
+        </is>
       </c>
       <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>47039</v>
-      </c>
-      <c r="B13" t="n">
-        <v>103160</v>
-      </c>
+        <v>45795</v>
+      </c>
+      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Hedgar Miralha Nascimento</t>
+          <t>Renato Rodzewics Silva</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
           <t>NAO</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
-        </is>
-      </c>
-      <c r="F13" t="n">
-        <v>1</v>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>ZONA NORTE,ZONA OESTE,ZONA LESTE,GUARULHOS</t>
+          <t>ZONA NORTE,ABCD,OSASCO-BARUERI-ALPHAVILLE</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>EFW3059</t>
-        </is>
-      </c>
-      <c r="L13" t="n">
-        <v>37026112821</v>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>46119496807</t>
+        </is>
       </c>
       <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>35339</v>
-      </c>
-      <c r="B14" t="n">
-        <v>52356</v>
-      </c>
+        <v>46454</v>
+      </c>
+      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
-          <t>João Victor Galdino Gonçalves</t>
+          <t>Caio da Silva Bezerra (Erick 2)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NAO</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1080,34 +1102,30 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>NAO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>OSASCO-BARUERI-ALPHAVILLE,ZONA NORTE,COTIA-EMBU-TABOAO</t>
+          <t>ZONA NORTE,ZONA OESTE,CENTRO</t>
         </is>
       </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>FVE0I20</t>
-        </is>
-      </c>
-      <c r="L14" t="n">
-        <v>44578842860</v>
-      </c>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>45795</v>
-      </c>
-      <c r="B15" t="inlineStr"/>
+        <v>47084</v>
+      </c>
+      <c r="B15" t="n">
+        <v>103182</v>
+      </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Renato Rodzewics Silva</t>
+          <t>Vinícius Oliveira Correia</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1125,30 +1143,38 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>NAO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>ZONA NORTE,ABCD,OSASCO-BARUERI-ALPHAVILLE</t>
+          <t>ZONA NORTE,ZONA OESTE,ZONA LESTE</t>
         </is>
       </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="n">
-        <v>46119496807</v>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>RUV9D51</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>34944268807</t>
+        </is>
       </c>
       <c r="M15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>46454</v>
-      </c>
-      <c r="B16" t="inlineStr"/>
+        <v>48907</v>
+      </c>
+      <c r="B16" t="n">
+        <v>104506</v>
+      </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Caio da Silva Bezerra (Erick 2)</t>
+          <t>Renato Forte</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1171,25 +1197,33 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>ZONA NORTE,ZONA OESTE,CENTRO</t>
+          <t>ZONA NORTE,CENTRO,ZONA LESTE,GUARULHOS</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ATW2C46</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>11496700880</t>
+        </is>
+      </c>
       <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>47084</v>
+        <v>48546</v>
       </c>
       <c r="B17" t="n">
-        <v>103182</v>
+        <v>104256</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Vinícius Oliveira Correia</t>
+          <t>Gabriel Ferreira de Souza</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1212,29 +1246,33 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>ZONA NORTE,ZONA OESTE,ZONA LESTE</t>
+          <t>ZONA NORTE,ZONA OESTE,OSASCO-BARUERI-ALPHAVILLE</t>
         </is>
       </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
-          <t>RUV9D51</t>
-        </is>
-      </c>
-      <c r="L17" t="n">
-        <v>34944268807</v>
+          <t>RTJ7E66</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>46065478806</t>
+        </is>
       </c>
       <c r="M17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>46474</v>
-      </c>
-      <c r="B18" t="inlineStr"/>
+        <v>47339</v>
+      </c>
+      <c r="B18" t="n">
+        <v>103339</v>
+      </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Ériclis Castro Nunes</t>
+          <t>Ricardo Barbosa do Nascimento</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1252,32 +1290,38 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>NAO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>CENTRO,ZONA OESTE,GUARULHOS</t>
+          <t>COTIA-EMBU-TABOAO,OSASCO-BARUERI-ALPHAVILLE,ZONA OESTE</t>
         </is>
       </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="n">
-        <v>43125943841</v>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>PUX6D34</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>31064536808</t>
+        </is>
       </c>
       <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>48547</v>
+        <v>31828</v>
       </c>
       <c r="B19" t="n">
-        <v>104257</v>
+        <v>22570</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Carlos Eduardo de Souza</t>
+          <t>Marcio Dell Aringa</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1300,36 +1344,38 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>ABCD,ZONA LESTE,ZONA SUL</t>
+          <t>ZONA LESTE,ABCD,ZONA NORTE</t>
         </is>
       </c>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
-          <t>GGO8B38</t>
-        </is>
-      </c>
-      <c r="L19" t="n">
-        <v>19277023805</v>
+          <t>NYA4J21</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>27466740847</t>
+        </is>
       </c>
       <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>48907</v>
+        <v>47424</v>
       </c>
       <c r="B20" t="n">
-        <v>104506</v>
+        <v>103406</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Renato Forte</t>
+          <t>Erick Gomes Oliveira - CARRO 2</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>NAO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1347,31 +1393,33 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>ZONA NORTE,CENTRO,ZONA LESTE,GUARULHOS</t>
+          <t>ZONA NORTE,ZONA OESTE,CENTRO</t>
         </is>
       </c>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>ATW2C46</t>
-        </is>
-      </c>
-      <c r="L20" t="n">
-        <v>11496700880</v>
+          <t>FVK3G29</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>47944413800</t>
+        </is>
       </c>
       <c r="M20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>48546</v>
+        <v>50016</v>
       </c>
       <c r="B21" t="n">
-        <v>104256</v>
+        <v>106040</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Gabriel Ferreira de Souza</t>
+          <t>Wellington Bittencourt dos Santos</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1394,36 +1442,40 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>ZONA NORTE,ZONA OESTE,OSASCO-BARUERI-ALPHAVILLE</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr"/>
+          <t>ZONA NORTE,ZONA OESTE,GUARULHOS</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>11984344347</v>
+      </c>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>RTJ7E66</t>
-        </is>
-      </c>
-      <c r="L21" t="n">
-        <v>46065478806</v>
+          <t>FUP1D50</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>22618919890</t>
+        </is>
       </c>
       <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>47339</v>
+        <v>46418</v>
       </c>
       <c r="B22" t="n">
-        <v>103339</v>
+        <v>102703</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Ricardo Barbosa do Nascimento</t>
+          <t>Jairo Domingues Abreu</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NAO</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1441,31 +1493,37 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>COTIA-EMBU-TABOAO,OSASCO-BARUERI-ALPHAVILLE,ZONA OESTE</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
+          <t>GUARULHOS,ZONA NORTE,CENTRO,ZONA LESTE</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>5511922305832</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>JairoAbreu@Freshlog.com</t>
+        </is>
+      </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>PUX6D34</t>
-        </is>
-      </c>
-      <c r="L22" t="n">
-        <v>31064536808</v>
+          <t>PXW0C92</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>41073933806</t>
+        </is>
       </c>
       <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>31828</v>
-      </c>
-      <c r="B23" t="n">
-        <v>22570</v>
-      </c>
+        <v>28438</v>
+      </c>
+      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Marcio Dell Aringa</t>
+          <t>Hugo Maçol Sousa (TESTE)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1475,11 +1533,11 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
+          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA,SABADO,DOMINGO</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1488,31 +1546,27 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>ZONA LESTE,ABCD,ZONA NORTE</t>
+          <t>ZONA NORTE,ZONA SUL,ZONA LESTE,ZONA OESTE,CENTRO,GUARULHOS,ABCD,OSASCO - BARUERI - SANTANA DE PARNAÍBA - ALPHAVILLE,COTIA - EMBU DAS ARTES - TABOÃO</t>
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>NYA4J21</t>
-        </is>
-      </c>
-      <c r="L23" t="n">
-        <v>27466740847</v>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>11111111111</t>
+        </is>
       </c>
       <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>47424</v>
-      </c>
-      <c r="B24" t="n">
-        <v>103406</v>
-      </c>
+        <v>50190</v>
+      </c>
+      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Erick Gomes Oliveira - CARRO 2</t>
+          <t>Samuel Fugazza Neto</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1535,31 +1589,33 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>ZONA NORTE,ZONA OESTE,CENTRO</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>FVK3G29</t>
-        </is>
-      </c>
-      <c r="L24" t="n">
-        <v>47944413800</v>
+          <t>ZONA NORTE,ZONA OESTE,ZONA SUL,ZONA LESTE</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>5511940851740</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>sn@freshlog.com.br</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>42993322885</t>
+        </is>
       </c>
       <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>50016</v>
-      </c>
-      <c r="B25" t="n">
-        <v>106040</v>
-      </c>
+        <v>50191</v>
+      </c>
+      <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Wellington Bittencourt dos Santos</t>
+          <t>Iago Mendes</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1582,38 +1638,40 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>ZONA NORTE,ZONA OESTE,GUARULHOS</t>
+          <t>ZONA NORTE,ZONA OESTE,ZONA SUL,ZONA LESTE</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>11984344347</v>
-      </c>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>FUP1D50</t>
-        </is>
-      </c>
-      <c r="L25" t="n">
-        <v>22618919890</v>
+        <v>5511970239954</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>im@freshlog.com.br</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>42640649884</t>
+        </is>
       </c>
       <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>46418</v>
+        <v>50199</v>
       </c>
       <c r="B26" t="n">
-        <v>102703</v>
+        <v>106175</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Jairo Domingues Abreu</t>
+          <t>Rafael Batista Ribeiro</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>NAO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1629,241 +1687,53 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>GUARULHOS,ZONA NORTE,CENTRO,ZONA LESTE</t>
-        </is>
-      </c>
+      <c r="H26" t="inlineStr"/>
       <c r="I26" t="n">
-        <v>5511922305832</v>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>JairoAbreu@Freshlog.com</t>
-        </is>
-      </c>
+        <v>11995109716</v>
+      </c>
+      <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
         <is>
-          <t>PXW0C92</t>
-        </is>
-      </c>
-      <c r="L26" t="n">
-        <v>41073933806</v>
-      </c>
-      <c r="M26" t="inlineStr"/>
+          <t>EMU6742</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>VAN_HR</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>28438</v>
+        <v>50258</v>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Hugo Maçol Sousa (TESTE)</t>
+          <t>LALAMOVE (virtual)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA,SABADO,DOMINGO</t>
-        </is>
-      </c>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
       <c r="F27" t="n">
-        <v>5</v>
+        <v>99</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>ZONA NORTE,ZONA SUL,ZONA LESTE,ZONA OESTE,CENTRO,GUARULHOS,ABCD,OSASCO - BARUERI - SANTANA DE PARNAÍBA - ALPHAVILLE,COTIA - EMBU DAS ARTES - TABOÃO</t>
-        </is>
-      </c>
+      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr"/>
-      <c r="L27" t="n">
-        <v>11111111111</v>
-      </c>
+      <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>50190</v>
-      </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Samuel Fugazza Neto</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
-        </is>
-      </c>
-      <c r="F28" t="n">
-        <v>1</v>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>ZONA NORTE,ZONA OESTE,ZONA SUL,ZONA LESTE</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>5511940851740</v>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>sn@freshlog.com.br</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="n">
-        <v>42993322885</v>
-      </c>
-      <c r="M28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>50191</v>
-      </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Iago Mendes</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
-        </is>
-      </c>
-      <c r="F29" t="n">
-        <v>1</v>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>ZONA NORTE,ZONA OESTE,ZONA SUL,ZONA LESTE</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>5511970239954</v>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>im@freshlog.com.br</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="n">
-        <v>42640649884</v>
-      </c>
-      <c r="M29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>50199</v>
-      </c>
-      <c r="B30" t="n">
-        <v>106175</v>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Rafael Batista Ribeiro</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
-        </is>
-      </c>
-      <c r="F30" t="n">
-        <v>1</v>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="n">
-        <v>11995109716</v>
-      </c>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>EMU6742</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>VAN_HR</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>50258</v>
-      </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>LALAMOVE (virtual)</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="n">
-        <v>99</v>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
BD_Motoristas: cadastra Diego Lopes (agente Vuupt 50219) como VUC
Pedido do Hugo (10/09, "Diego Pego" = Diego Lopes na Vuupt). Seg-Sex,
1 rota/dia, todas as zonas, telefone/e-mail/CPF vindos do agente Vuupt.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/BD_MOTORISTAS.xlsx
+++ b/dados/BD_MOTORISTAS.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M27"/>
+  <dimension ref="A1:M28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1735,6 +1735,59 @@
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
     </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>50219</v>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Diego Lopes</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>ZONA NORTE,ZONA SUL,ZONA LESTE,ZONA OESTE,CENTRO,GUARULHOS,ABCD,OSASCO-BARUERI-ALPHAVILLE,COTIA-EMBU-TABOAO</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>5511982838487</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>dl@freshlog.com.br</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>38411793800</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>VUC</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
BD_Motoristas: cadastra Patricia Alexandre da Silva (agente Vuupt 46379) como VAN_HR, seg-sex, 9 zonas, aceita viagens
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/BD_MOTORISTAS.xlsx
+++ b/dados/BD_MOTORISTAS.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,71 +413,71 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M28"/>
+  <dimension ref="A1:M29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>AGENT_ID_VUUPT</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>VEHICLE_ID_VUUPT</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>NOME_MOTORISTA</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>ACEITA_VIAGENS</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>DIAS_DISPONIVEIS</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>MAX_ROTAS_DIA</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>ATIVO</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>ZONAS_PREFERIDAS</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>TELEFONE_MOTORISTA</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>EMAIL_MOTORISTA</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>PLACA</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>CPF_MOTORISTA</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>TIPO_VEICULO</t>
         </is>
@@ -1788,6 +1776,49 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>46379</v>
+      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Patrícia Alexandre da Silva</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>ZONA NORTE,ZONA SUL,ZONA LESTE,ZONA OESTE,CENTRO,GUARULHOS,ABCD,OSASCO-BARUERI-ALPHAVILLE,COTIA-EMBU-TABOAO</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>VAN_HR</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Motoristas: cadastra Marlon (31861) e Maisa (50826) na planilha
Marlon Augusto Ribeiro Pumes: Zona Sul/Norte/Oeste/Leste, aceita viagens, Seg-Sex, max 1.
Maisa de Souza Leroz Silva: mesmas zonas, nao aceita viagens, Seg-Sex, max 1, Fiorino (TIPO_VEICULO vazio, so veiculo grande usa a coluna).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/BD_MOTORISTAS.xlsx
+++ b/dados/BD_MOTORISTAS.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,71 +425,71 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M29"/>
+  <dimension ref="A1:M31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>AGENT_ID_VUUPT</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>VEHICLE_ID_VUUPT</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>NOME_MOTORISTA</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>ACEITA_VIAGENS</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>DIAS_DISPONIVEIS</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>MAX_ROTAS_DIA</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>ATIVO</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>ZONAS_PREFERIDAS</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>TELEFONE_MOTORISTA</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>EMAIL_MOTORISTA</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>PLACA</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>CPF_MOTORISTA</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>TIPO_VEICULO</t>
         </is>
@@ -1819,6 +1831,84 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>31861</v>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Marlon Augusto Ribeiro Pumes</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>ZONA SUL,ZONA NORTE,ZONA OESTE,ZONA LESTE</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>50826</v>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Maisa de Souza Leroz Silva</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>ZONA SUL,ZONA NORTE,ZONA OESTE,ZONA LESTE</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Motoristas: TIPO_VEICULO preenchido com FIORINO nos 25 sem carro
So a coluna TIPO_VEICULO das celulas vazias; LALAMOVE (virtual) e o
cadastro de teste ficaram em branco de proposito. Hugo, 22/09.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/BD_MOTORISTAS.xlsx
+++ b/dados/BD_MOTORISTAS.xlsx
@@ -530,8 +530,6 @@
           <t>ZONA NORTE,GUARULHOS,ZONA LESTE</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
           <t>PZD7G26</t>
@@ -542,7 +540,11 @@
           <t>13415403831</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>FIORINO</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -579,8 +581,6 @@
           <t>ZONA NORTE</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
           <t>OQH7B64</t>
@@ -591,7 +591,11 @@
           <t>34822303829</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>FIORINO</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -628,8 +632,6 @@
           <t>ZONA NORTE,ABCD,COTIA-EMBU-TABOAO</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
           <t>EZD9B14</t>
@@ -640,7 +642,11 @@
           <t>9474142742</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>FIORINO</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -677,8 +683,6 @@
           <t>OSASCO-BARUERI-ALPHAVILLE,ABCD,GUARULHOS</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
           <t>FAW8I34</t>
@@ -689,7 +693,11 @@
           <t>28090589898</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>FIORINO</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -726,8 +734,6 @@
           <t>ZONA NORTE,ZONA OESTE,CENTRO</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
           <t>EDY1E57</t>
@@ -738,7 +744,11 @@
           <t>47944413800</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>FIORINO</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -775,8 +785,6 @@
           <t>GUARULHOS,ZONA NORTE,ZONA LESTE,ABCD</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>FYD1E68</t>
@@ -787,7 +795,11 @@
           <t>30700585826</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>FIORINO</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -824,8 +836,6 @@
           <t>ZONA NORTE,CENTRO,ZONA OESTE,ZONA SUL</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>EAA0985</t>
@@ -836,7 +846,11 @@
           <t>22425592814</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>FIORINO</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -873,8 +887,6 @@
           <t>ZONA OESTE,ZONA NORTE,CENTRO</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>FQJ7F16</t>
@@ -885,7 +897,11 @@
           <t>38938114864</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>FIORINO</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -922,8 +938,6 @@
           <t>ZONA LESTE,GUARULHOS,ABCD</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
           <t xml:space="preserve">PWI9H55 </t>
@@ -934,7 +948,11 @@
           <t>28209297880</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>FIORINO</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -971,8 +989,6 @@
           <t>ZONA NORTE,ZONA OESTE,ZONA LESTE,GUARULHOS</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
           <t>EFW3059</t>
@@ -983,7 +999,11 @@
           <t>37026112821</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>FIORINO</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1020,8 +1040,6 @@
           <t>OSASCO-BARUERI-ALPHAVILLE,ZONA NORTE,COTIA-EMBU-TABOAO</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
           <t>FVE0I20</t>
@@ -1032,13 +1050,16 @@
           <t>44578842860</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr"/>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>FIORINO</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
         <v>45795</v>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>Renato Rodzewics Silva</t>
@@ -1067,21 +1088,21 @@
           <t>ZONA NORTE,ABCD,OSASCO-BARUERI-ALPHAVILLE</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
           <t>46119496807</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr"/>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>FIORINO</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
         <v>46454</v>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>Caio da Silva Bezerra (Erick 2)</t>
@@ -1110,11 +1131,11 @@
           <t>ZONA NORTE,ZONA OESTE,CENTRO</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>FIORINO</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1151,8 +1172,6 @@
           <t>ZONA NORTE,ZONA OESTE,ZONA LESTE</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
           <t>RUV9D51</t>
@@ -1163,7 +1182,11 @@
           <t>34944268807</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>FIORINO</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1200,8 +1223,6 @@
           <t>ZONA NORTE,CENTRO,ZONA LESTE,GUARULHOS</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
           <t>ATW2C46</t>
@@ -1212,7 +1233,11 @@
           <t>11496700880</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>FIORINO</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1249,8 +1274,6 @@
           <t>ZONA NORTE,ZONA OESTE,OSASCO-BARUERI-ALPHAVILLE</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
           <t>RTJ7E66</t>
@@ -1261,7 +1284,11 @@
           <t>46065478806</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>FIORINO</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1298,8 +1325,6 @@
           <t>COTIA-EMBU-TABOAO,OSASCO-BARUERI-ALPHAVILLE,ZONA OESTE</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
           <t>PUX6D34</t>
@@ -1310,7 +1335,11 @@
           <t>31064536808</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr"/>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>FIORINO</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1347,8 +1376,6 @@
           <t>ZONA LESTE,ABCD,ZONA NORTE</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
           <t>NYA4J21</t>
@@ -1359,7 +1386,11 @@
           <t>27466740847</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr"/>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>FIORINO</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1396,8 +1427,6 @@
           <t>ZONA NORTE,ZONA OESTE,CENTRO</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
           <t>FVK3G29</t>
@@ -1408,7 +1437,11 @@
           <t>47944413800</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr"/>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>FIORINO</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1448,7 +1481,6 @@
       <c r="I21" t="n">
         <v>11984344347</v>
       </c>
-      <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
           <t>FUP1D50</t>
@@ -1459,7 +1491,11 @@
           <t>22618919890</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>FIORINO</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1514,13 +1550,16 @@
           <t>41073933806</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr"/>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>FIORINO</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
         <v>28438</v>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
           <t>Hugo Maçol Sousa (TESTE)</t>
@@ -1549,21 +1588,16 @@
           <t>ZONA NORTE,ZONA SUL,ZONA LESTE,ZONA OESTE,CENTRO,GUARULHOS,ABCD,OSASCO - BARUERI - SANTANA DE PARNAÍBA - ALPHAVILLE,COTIA - EMBU DAS ARTES - TABOÃO</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
           <t>11111111111</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
         <v>50190</v>
       </c>
-      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
           <t>Samuel Fugazza Neto</t>
@@ -1600,19 +1634,21 @@
           <t>sn@freshlog.com.br</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
           <t>42993322885</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr"/>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>FIORINO</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
         <v>50191</v>
       </c>
-      <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
           <t>Iago Mendes</t>
@@ -1649,13 +1685,16 @@
           <t>im@freshlog.com.br</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
           <t>42640649884</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr"/>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>FIORINO</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1687,17 +1726,14 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
       <c r="I26" t="n">
         <v>11995109716</v>
       </c>
-      <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
         <is>
           <t>EMU6742</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr">
         <is>
           <t>VAN_HR</t>
@@ -1708,7 +1744,6 @@
       <c r="A27" t="n">
         <v>50258</v>
       </c>
-      <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
           <t>LALAMOVE (virtual)</t>
@@ -1719,7 +1754,6 @@
           <t>NAO</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="n">
         <v>99</v>
       </c>
@@ -1728,18 +1762,11 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
         <v>50219</v>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
           <t>Diego Lopes</t>
@@ -1776,7 +1803,6 @@
           <t>dl@freshlog.com.br</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
           <t>38411793800</t>
@@ -1792,7 +1818,6 @@
       <c r="A29" t="n">
         <v>46379</v>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
           <t>Patrícia Alexandre da Silva</t>
@@ -1821,10 +1846,6 @@
           <t>ZONA NORTE,ZONA SUL,ZONA LESTE,ZONA OESTE,CENTRO,GUARULHOS,ABCD,OSASCO-BARUERI-ALPHAVILLE,COTIA-EMBU-TABOAO</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr">
         <is>
           <t>VAN_HR</t>
@@ -1835,7 +1856,6 @@
       <c r="A30" t="n">
         <v>31861</v>
       </c>
-      <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
           <t>Marlon Augusto Ribeiro Pumes</t>
@@ -1864,17 +1884,16 @@
           <t>ZONA SUL,ZONA NORTE,ZONA OESTE,ZONA LESTE</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>FIORINO</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
         <v>50826</v>
       </c>
-      <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
           <t>Maisa de Souza Leroz Silva</t>
@@ -1903,11 +1922,11 @@
           <t>ZONA SUL,ZONA NORTE,ZONA OESTE,ZONA LESTE</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>FIORINO</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Motoristas: cadastro de teste inativo e zonas padrao pro Rafael
Hugo Macol Sousa (TESTE, 28438) estava ATIVO=SIM com 5 rotas/dia em
todas as zonas -- elegivel a rota real. Rafael Batista Ribeiro (VAN/HR)
estava com ZONAS_PREFERIDAS vazio e nunca era escolhido; recebe o
padrao Norte, Sul, Leste e Oeste. Pedido do Hugo, 23/09.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/BD_MOTORISTAS.xlsx
+++ b/dados/BD_MOTORISTAS.xlsx
@@ -1580,7 +1580,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NAO</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1724,6 +1724,11 @@
       <c r="G26" t="inlineStr">
         <is>
           <t>SIM</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>ZONA NORTE,ZONA SUL,ZONA LESTE,ZONA OESTE</t>
         </is>
       </c>
       <c r="I26" t="n">

</xml_diff>

<commit_message>
Motoristas: sabado nos dias de Erick, Caio, Maisa, Ricardo e Vinicius
Com o cadastro de teste inativo, nenhum motorista real tinha sabado e
toda rota de sabado saia sem motorista. As duas linhas do Erick (mesmo
agent_id) recebem o sabado. Pedido do Hugo, 23/09.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/BD_MOTORISTAS.xlsx
+++ b/dados/BD_MOTORISTAS.xlsx
@@ -718,7 +718,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
+          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA,SABADO</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
+          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA,SABADO</t>
         </is>
       </c>
       <c r="F14" t="n">
@@ -1156,7 +1156,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
+          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA,SABADO</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -1309,7 +1309,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
+          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA,SABADO</t>
         </is>
       </c>
       <c r="F18" t="n">
@@ -1411,7 +1411,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
+          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA,SABADO</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -1911,7 +1911,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
+          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA,SABADO</t>
         </is>
       </c>
       <c r="F31" t="n">

</xml_diff>

<commit_message>
Motoristas: exclui a linha duplicada Erick - CARRO 2
Mesmo agent_id da linha principal, mas com ACEITA_VIAGENS=SIM enquanto a
principal diz NAO -- o Erick recebia viagem pela linha duplicada.
Pedido do Hugo, 23/09.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/BD_MOTORISTAS.xlsx
+++ b/dados/BD_MOTORISTAS.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M31"/>
+  <dimension ref="A1:M30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1394,14 +1394,14 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>47424</v>
+        <v>50016</v>
       </c>
       <c r="B20" t="n">
-        <v>103406</v>
+        <v>106040</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Erick Gomes Oliveira - CARRO 2</t>
+          <t>Wellington Bittencourt dos Santos</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1411,7 +1411,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA,SABADO</t>
+          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -1424,17 +1424,20 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>ZONA NORTE,ZONA OESTE,CENTRO</t>
-        </is>
+          <t>ZONA NORTE,ZONA OESTE,GUARULHOS</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>11984344347</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>FVK3G29</t>
+          <t>FUP1D50</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>47944413800</t>
+          <t>22618919890</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1445,19 +1448,19 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>50016</v>
+        <v>46418</v>
       </c>
       <c r="B21" t="n">
-        <v>106040</v>
+        <v>102703</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Wellington Bittencourt dos Santos</t>
+          <t>Jairo Domingues Abreu</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NAO</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1475,20 +1478,25 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>ZONA NORTE,ZONA OESTE,GUARULHOS</t>
+          <t>GUARULHOS,ZONA NORTE,CENTRO,ZONA LESTE</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>11984344347</v>
+        <v>5511922305832</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>JairoAbreu@Freshlog.com</t>
+        </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>FUP1D50</t>
+          <t>PXW0C92</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>22618919890</t>
+          <t>41073933806</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1499,70 +1507,49 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>46418</v>
-      </c>
-      <c r="B22" t="n">
-        <v>102703</v>
+        <v>28438</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Jairo Domingues Abreu</t>
+          <t>Hugo Maçol Sousa (TESTE)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA,SABADO,DOMINGO</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>5</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
           <t>NAO</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
-        </is>
-      </c>
-      <c r="F22" t="n">
-        <v>1</v>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>GUARULHOS,ZONA NORTE,CENTRO,ZONA LESTE</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>5511922305832</v>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>JairoAbreu@Freshlog.com</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>PXW0C92</t>
+          <t>ZONA NORTE,ZONA SUL,ZONA LESTE,ZONA OESTE,CENTRO,GUARULHOS,ABCD,OSASCO - BARUERI - SANTANA DE PARNAÍBA - ALPHAVILLE,COTIA - EMBU DAS ARTES - TABOÃO</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>41073933806</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>FIORINO</t>
+          <t>11111111111</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>28438</v>
+        <v>50190</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Hugo Maçol Sousa (TESTE)</t>
+          <t>Samuel Fugazza Neto</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1572,35 +1559,48 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA,SABADO,DOMINGO</t>
+          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>NAO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>ZONA NORTE,ZONA SUL,ZONA LESTE,ZONA OESTE,CENTRO,GUARULHOS,ABCD,OSASCO - BARUERI - SANTANA DE PARNAÍBA - ALPHAVILLE,COTIA - EMBU DAS ARTES - TABOÃO</t>
+          <t>ZONA NORTE,ZONA OESTE,ZONA SUL,ZONA LESTE</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>5511940851740</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>sn@freshlog.com.br</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>11111111111</t>
+          <t>42993322885</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>FIORINO</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>50190</v>
+        <v>50191</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Samuel Fugazza Neto</t>
+          <t>Iago Mendes</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1627,16 +1627,16 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>5511940851740</v>
+        <v>5511970239954</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>sn@freshlog.com.br</t>
+          <t>im@freshlog.com.br</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>42993322885</t>
+          <t>42640649884</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -1647,11 +1647,14 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>50191</v>
+        <v>50199</v>
+      </c>
+      <c r="B25" t="n">
+        <v>106175</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Iago Mendes</t>
+          <t>Rafael Batista Ribeiro</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1674,107 +1677,104 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>ZONA NORTE,ZONA OESTE,ZONA SUL,ZONA LESTE</t>
+          <t>ZONA NORTE,ZONA SUL,ZONA LESTE,ZONA OESTE</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>5511970239954</v>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>im@freshlog.com.br</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>42640649884</t>
+        <v>11995109716</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>EMU6742</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>FIORINO</t>
+          <t>VAN_HR</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>50199</v>
-      </c>
-      <c r="B26" t="n">
-        <v>106175</v>
+        <v>50258</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Rafael Batista Ribeiro</t>
+          <t>LALAMOVE (virtual)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
+          <t>NAO</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>1</v>
+        <v>99</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
           <t>SIM</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>ZONA NORTE,ZONA SUL,ZONA LESTE,ZONA OESTE</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>11995109716</v>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>EMU6742</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>VAN_HR</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>50258</v>
+        <v>50219</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>LALAMOVE (virtual)</t>
+          <t>Diego Lopes</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>NAO</t>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>99</v>
+        <v>1</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
           <t>SIM</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>ZONA NORTE,ZONA SUL,ZONA LESTE,ZONA OESTE,CENTRO,GUARULHOS,ABCD,OSASCO-BARUERI-ALPHAVILLE,COTIA-EMBU-TABOAO</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>5511982838487</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>dl@freshlog.com.br</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>38411793800</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>VUC</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>50219</v>
+        <v>46379</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Diego Lopes</t>
+          <t>Patrícia Alexandre da Silva</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1800,32 +1800,19 @@
           <t>ZONA NORTE,ZONA SUL,ZONA LESTE,ZONA OESTE,CENTRO,GUARULHOS,ABCD,OSASCO-BARUERI-ALPHAVILLE,COTIA-EMBU-TABOAO</t>
         </is>
       </c>
-      <c r="I28" t="n">
-        <v>5511982838487</v>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>dl@freshlog.com.br</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>38411793800</t>
-        </is>
-      </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>VUC</t>
+          <t>VAN_HR</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>46379</v>
+        <v>31861</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Patrícia Alexandre da Silva</t>
+          <t>Marlon Augusto Ribeiro Pumes</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1848,32 +1835,32 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>ZONA NORTE,ZONA SUL,ZONA LESTE,ZONA OESTE,CENTRO,GUARULHOS,ABCD,OSASCO-BARUERI-ALPHAVILLE,COTIA-EMBU-TABOAO</t>
+          <t>ZONA SUL,ZONA NORTE,ZONA OESTE,ZONA LESTE</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>VAN_HR</t>
+          <t>FIORINO</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>31861</v>
+        <v>50826</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Marlon Augusto Ribeiro Pumes</t>
+          <t>Maisa de Souza Leroz Silva</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NAO</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
+          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA,SABADO</t>
         </is>
       </c>
       <c r="F30" t="n">
@@ -1890,44 +1877,6 @@
         </is>
       </c>
       <c r="M30" t="inlineStr">
-        <is>
-          <t>FIORINO</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>50826</v>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Maisa de Souza Leroz Silva</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>NAO</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA,SABADO</t>
-        </is>
-      </c>
-      <c r="F31" t="n">
-        <v>1</v>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>ZONA SUL,ZONA NORTE,ZONA OESTE,ZONA LESTE</t>
-        </is>
-      </c>
-      <c r="M31" t="inlineStr">
         <is>
           <t>FIORINO</t>
         </is>

</xml_diff>

<commit_message>
Motoristas: CPF do Clayson com o zero a esquerda
Estava digitado com 10 digitos (sem o 0 inicial) e o catalogo tratava
como sem CPF -- ele nao aparecia na identificacao por CPF (marketplace
e app). Gravado como texto. CPF passado pelo Hugo, 23/09.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/BD_MOTORISTAS.xlsx
+++ b/dados/BD_MOTORISTAS.xlsx
@@ -55,11 +55,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -637,9 +638,9 @@
           <t>EZD9B14</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>9474142742</t>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>09474142742</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">

</xml_diff>

<commit_message>
Motoristas: Samuel inativo, Fagner so carga seca, placa da Maisa
Samuel Fugazza Neto ATIVO=NAO; Fagner Macedo APENAS_CARGA_SECA=SIM
(coluna nova); Maisa PLACA=GDI5A39 (estava vazia, entra na trava de
rodizio). Pedido do Hugo, 23/09.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/BD_MOTORISTAS.xlsx
+++ b/dados/BD_MOTORISTAS.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M30"/>
+  <dimension ref="A1:N30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -495,6 +495,11 @@
           <t>TIPO_VEICULO</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>APENAS_CARGA_SECA</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -903,6 +908,11 @@
           <t>FIORINO</t>
         </is>
       </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1568,7 +1578,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NAO</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1875,6 +1885,11 @@
       <c r="H30" t="inlineStr">
         <is>
           <t>ZONA SUL,ZONA NORTE,ZONA OESTE,ZONA LESTE</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>GDI5A39</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">

</xml_diff>

<commit_message>
Motoristas: placa do Marlon
RMZ1B04 (estava vazia, entra na trava de rodizio). Pedido do Hugo, 23/09.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/BD_MOTORISTAS.xlsx
+++ b/dados/BD_MOTORISTAS.xlsx
@@ -1849,6 +1849,11 @@
           <t>ZONA SUL,ZONA NORTE,ZONA OESTE,ZONA LESTE</t>
         </is>
       </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>RMZ1B04</t>
+        </is>
+      </c>
       <c r="M29" t="inlineStr">
         <is>
           <t>FIORINO</t>

</xml_diff>

<commit_message>
Motoristas: veiculo grande so pega rota do proprio porte + planilha (2 VAN_HR, 3 inativos)
Regra (Hugo, 25/09): motorista que nao e Fiorino so e elegivel pra rota
classificada com o porte exato do carro dele (VAN_HR so VAN_HR, VUC so
VUC...). Nem rota comum, nem porte menor -- acabou o "maior cobre menor"
de veiculo_comporta. Fiorino e motorista sem tipo seguem so na rota comum.

Planilha: Joao Victor e Renato Rodzewics viram VAN_HR; Erivan, Jairo e
Adriano Alves inativados.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/BD_MOTORISTAS.xlsx
+++ b/dados/BD_MOTORISTAS.xlsx
@@ -55,12 +55,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -495,7 +494,7 @@
           <t>TIPO_VEICULO</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>APENAS_CARGA_SECA</t>
         </is>
@@ -528,7 +527,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NAO</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -536,6 +535,8 @@
           <t>ZONA NORTE,GUARULHOS,ZONA LESTE</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
           <t>PZD7G26</t>
@@ -551,6 +552,7 @@
           <t>FIORINO</t>
         </is>
       </c>
+      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -587,6 +589,8 @@
           <t>ZONA NORTE</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
           <t>OQH7B64</t>
@@ -602,6 +606,7 @@
           <t>FIORINO</t>
         </is>
       </c>
+      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -638,12 +643,14 @@
           <t>ZONA NORTE,ABCD,COTIA-EMBU-TABOAO</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
           <t>EZD9B14</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>09474142742</t>
         </is>
@@ -653,6 +660,7 @@
           <t>FIORINO</t>
         </is>
       </c>
+      <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -689,6 +697,8 @@
           <t>OSASCO-BARUERI-ALPHAVILLE,ABCD,GUARULHOS</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
           <t>FAW8I34</t>
@@ -704,6 +714,7 @@
           <t>FIORINO</t>
         </is>
       </c>
+      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -740,6 +751,8 @@
           <t>ZONA NORTE,ZONA OESTE,CENTRO</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
           <t>EDY1E57</t>
@@ -755,6 +768,7 @@
           <t>FIORINO</t>
         </is>
       </c>
+      <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -783,7 +797,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NAO</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -791,6 +805,8 @@
           <t>GUARULHOS,ZONA NORTE,ZONA LESTE,ABCD</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>FYD1E68</t>
@@ -806,6 +822,7 @@
           <t>FIORINO</t>
         </is>
       </c>
+      <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -842,6 +859,8 @@
           <t>ZONA NORTE,CENTRO,ZONA OESTE,ZONA SUL</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>EAA0985</t>
@@ -857,6 +876,7 @@
           <t>FIORINO</t>
         </is>
       </c>
+      <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -893,6 +913,8 @@
           <t>ZONA OESTE,ZONA NORTE,CENTRO</t>
         </is>
       </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>FQJ7F16</t>
@@ -949,6 +971,8 @@
           <t>ZONA LESTE,GUARULHOS,ABCD</t>
         </is>
       </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
           <t xml:space="preserve">PWI9H55 </t>
@@ -964,6 +988,7 @@
           <t>FIORINO</t>
         </is>
       </c>
+      <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1000,6 +1025,8 @@
           <t>ZONA NORTE,ZONA OESTE,ZONA LESTE,GUARULHOS</t>
         </is>
       </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
           <t>EFW3059</t>
@@ -1015,6 +1042,7 @@
           <t>FIORINO</t>
         </is>
       </c>
+      <c r="N11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1051,6 +1079,8 @@
           <t>OSASCO-BARUERI-ALPHAVILLE,ZONA NORTE,COTIA-EMBU-TABOAO</t>
         </is>
       </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
           <t>FVE0I20</t>
@@ -1063,14 +1093,16 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>FIORINO</t>
-        </is>
-      </c>
+          <t>VAN_HR</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
         <v>45795</v>
       </c>
+      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>Renato Rodzewics Silva</t>
@@ -1099,6 +1131,9 @@
           <t>ZONA NORTE,ABCD,OSASCO-BARUERI-ALPHAVILLE</t>
         </is>
       </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
           <t>46119496807</t>
@@ -1106,14 +1141,16 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>FIORINO</t>
-        </is>
-      </c>
+          <t>VAN_HR</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
         <v>46454</v>
       </c>
+      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>Caio da Silva Bezerra (Erick 2)</t>
@@ -1142,11 +1179,16 @@
           <t>ZONA NORTE,ZONA OESTE,CENTRO</t>
         </is>
       </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
           <t>FIORINO</t>
         </is>
       </c>
+      <c r="N14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1183,6 +1225,8 @@
           <t>ZONA NORTE,ZONA OESTE,ZONA LESTE</t>
         </is>
       </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
           <t>RUV9D51</t>
@@ -1198,6 +1242,7 @@
           <t>FIORINO</t>
         </is>
       </c>
+      <c r="N15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1234,6 +1279,8 @@
           <t>ZONA NORTE,CENTRO,ZONA LESTE,GUARULHOS</t>
         </is>
       </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
           <t>ATW2C46</t>
@@ -1249,6 +1296,7 @@
           <t>FIORINO</t>
         </is>
       </c>
+      <c r="N16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1285,6 +1333,8 @@
           <t>ZONA NORTE,ZONA OESTE,OSASCO-BARUERI-ALPHAVILLE</t>
         </is>
       </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
           <t>RTJ7E66</t>
@@ -1300,6 +1350,7 @@
           <t>FIORINO</t>
         </is>
       </c>
+      <c r="N17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1336,6 +1387,8 @@
           <t>COTIA-EMBU-TABOAO,OSASCO-BARUERI-ALPHAVILLE,ZONA OESTE</t>
         </is>
       </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
           <t>PUX6D34</t>
@@ -1351,6 +1404,7 @@
           <t>FIORINO</t>
         </is>
       </c>
+      <c r="N18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1387,6 +1441,8 @@
           <t>ZONA LESTE,ABCD,ZONA NORTE</t>
         </is>
       </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
           <t>NYA4J21</t>
@@ -1402,6 +1458,7 @@
           <t>FIORINO</t>
         </is>
       </c>
+      <c r="N19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1441,6 +1498,7 @@
       <c r="I20" t="n">
         <v>11984344347</v>
       </c>
+      <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
           <t>FUP1D50</t>
@@ -1456,6 +1514,7 @@
           <t>FIORINO</t>
         </is>
       </c>
+      <c r="N20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1484,7 +1543,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NAO</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1515,11 +1574,13 @@
           <t>FIORINO</t>
         </is>
       </c>
+      <c r="N21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
         <v>28438</v>
       </c>
+      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
           <t>Hugo Maçol Sousa (TESTE)</t>
@@ -1548,16 +1609,22 @@
           <t>ZONA NORTE,ZONA SUL,ZONA LESTE,ZONA OESTE,CENTRO,GUARULHOS,ABCD,OSASCO - BARUERI - SANTANA DE PARNAÍBA - ALPHAVILLE,COTIA - EMBU DAS ARTES - TABOÃO</t>
         </is>
       </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
           <t>11111111111</t>
         </is>
       </c>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
         <v>50190</v>
       </c>
+      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
           <t>Samuel Fugazza Neto</t>
@@ -1594,6 +1661,7 @@
           <t>sn@freshlog.com.br</t>
         </is>
       </c>
+      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
           <t>42993322885</t>
@@ -1604,11 +1672,13 @@
           <t>FIORINO</t>
         </is>
       </c>
+      <c r="N23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
         <v>50191</v>
       </c>
+      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
           <t>Iago Mendes</t>
@@ -1645,6 +1715,7 @@
           <t>im@freshlog.com.br</t>
         </is>
       </c>
+      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
           <t>42640649884</t>
@@ -1655,6 +1726,7 @@
           <t>FIORINO</t>
         </is>
       </c>
+      <c r="N24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1694,21 +1766,25 @@
       <c r="I25" t="n">
         <v>11995109716</v>
       </c>
+      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
           <t>EMU6742</t>
         </is>
       </c>
+      <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr">
         <is>
           <t>VAN_HR</t>
         </is>
       </c>
+      <c r="N25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
         <v>50258</v>
       </c>
+      <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
           <t>LALAMOVE (virtual)</t>
@@ -1719,6 +1795,7 @@
           <t>NAO</t>
         </is>
       </c>
+      <c r="E26" t="inlineStr"/>
       <c r="F26" t="n">
         <v>99</v>
       </c>
@@ -1727,11 +1804,19 @@
           <t>SIM</t>
         </is>
       </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
         <v>50219</v>
       </c>
+      <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
           <t>Diego Lopes</t>
@@ -1768,6 +1853,7 @@
           <t>dl@freshlog.com.br</t>
         </is>
       </c>
+      <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
           <t>38411793800</t>
@@ -1778,11 +1864,13 @@
           <t>VUC</t>
         </is>
       </c>
+      <c r="N27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
         <v>46379</v>
       </c>
+      <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
           <t>Patrícia Alexandre da Silva</t>
@@ -1811,16 +1899,22 @@
           <t>ZONA NORTE,ZONA SUL,ZONA LESTE,ZONA OESTE,CENTRO,GUARULHOS,ABCD,OSASCO-BARUERI-ALPHAVILLE,COTIA-EMBU-TABOAO</t>
         </is>
       </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr">
         <is>
           <t>VAN_HR</t>
         </is>
       </c>
+      <c r="N28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
         <v>31861</v>
       </c>
+      <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
           <t>Marlon Augusto Ribeiro Pumes</t>
@@ -1849,21 +1943,26 @@
           <t>ZONA SUL,ZONA NORTE,ZONA OESTE,ZONA LESTE</t>
         </is>
       </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr">
         <is>
           <t>RMZ1B04</t>
         </is>
       </c>
+      <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr">
         <is>
           <t>FIORINO</t>
         </is>
       </c>
+      <c r="N29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
         <v>50826</v>
       </c>
+      <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
           <t>Maisa de Souza Leroz Silva</t>
@@ -1892,16 +1991,20 @@
           <t>ZONA SUL,ZONA NORTE,ZONA OESTE,ZONA LESTE</t>
         </is>
       </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
           <t>GDI5A39</t>
         </is>
       </c>
+      <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr">
         <is>
           <t>FIORINO</t>
         </is>
       </c>
+      <c r="N30" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Motoristas: cadastro do Rafael de Morais Coelho (agent 51410)
FIORINO placa RFK1H77, seg a sex, zonas Norte/Sul/Leste/Oeste, 1 rota/dia,
ativo. CPF 31880016818 (tambem e a chave PIX dele). Sem VEHICLE_ID_VUUPT.
Pedido do Hugo, 01/10.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q9cCgX2j2P6BUmLBbUFnNB
</commit_message>
<xml_diff>
--- a/dados/BD_MOTORISTAS.xlsx
+++ b/dados/BD_MOTORISTAS.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N30"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -535,8 +535,6 @@
           <t>ZONA NORTE,GUARULHOS,ZONA LESTE</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
           <t>PZD7G26</t>
@@ -552,7 +550,6 @@
           <t>FIORINO</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -589,8 +586,6 @@
           <t>ZONA NORTE</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
           <t>OQH7B64</t>
@@ -606,7 +601,6 @@
           <t>FIORINO</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -643,8 +637,6 @@
           <t>ZONA NORTE,ABCD,COTIA-EMBU-TABOAO</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
           <t>EZD9B14</t>
@@ -660,7 +652,6 @@
           <t>FIORINO</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -697,8 +688,6 @@
           <t>OSASCO-BARUERI-ALPHAVILLE,ABCD,GUARULHOS</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
           <t>FAW8I34</t>
@@ -714,7 +703,6 @@
           <t>FIORINO</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -751,8 +739,6 @@
           <t>ZONA NORTE,ZONA OESTE,CENTRO</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
           <t>EDY1E57</t>
@@ -768,7 +754,6 @@
           <t>FIORINO</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -805,8 +790,6 @@
           <t>GUARULHOS,ZONA NORTE,ZONA LESTE,ABCD</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>FYD1E68</t>
@@ -822,7 +805,6 @@
           <t>FIORINO</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -859,8 +841,6 @@
           <t>ZONA NORTE,CENTRO,ZONA OESTE,ZONA SUL</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>EAA0985</t>
@@ -876,7 +856,6 @@
           <t>FIORINO</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -913,8 +892,6 @@
           <t>ZONA OESTE,ZONA NORTE,CENTRO</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>FQJ7F16</t>
@@ -971,8 +948,6 @@
           <t>ZONA LESTE,GUARULHOS,ABCD</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
           <t xml:space="preserve">PWI9H55 </t>
@@ -988,7 +963,6 @@
           <t>FIORINO</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1025,8 +999,6 @@
           <t>ZONA NORTE,ZONA OESTE,ZONA LESTE,GUARULHOS</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
           <t>EFW3059</t>
@@ -1042,7 +1014,6 @@
           <t>FIORINO</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1079,8 +1050,6 @@
           <t>OSASCO-BARUERI-ALPHAVILLE,ZONA NORTE,COTIA-EMBU-TABOAO</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
           <t>FVE0I20</t>
@@ -1096,13 +1065,11 @@
           <t>VAN_HR</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
         <v>45795</v>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>Renato Rodzewics Silva</t>
@@ -1131,9 +1098,6 @@
           <t>ZONA NORTE,ABCD,OSASCO-BARUERI-ALPHAVILLE</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
           <t>46119496807</t>
@@ -1144,13 +1108,11 @@
           <t>VAN_HR</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
         <v>46454</v>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>Caio da Silva Bezerra (Erick 2)</t>
@@ -1179,16 +1141,11 @@
           <t>ZONA NORTE,ZONA OESTE,CENTRO</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
           <t>FIORINO</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1225,8 +1182,6 @@
           <t>ZONA NORTE,ZONA OESTE,ZONA LESTE</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
           <t>RUV9D51</t>
@@ -1242,7 +1197,6 @@
           <t>FIORINO</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1279,8 +1233,6 @@
           <t>ZONA NORTE,CENTRO,ZONA LESTE,GUARULHOS</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
           <t>ATW2C46</t>
@@ -1296,7 +1248,6 @@
           <t>FIORINO</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1333,8 +1284,6 @@
           <t>ZONA NORTE,ZONA OESTE,OSASCO-BARUERI-ALPHAVILLE</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
           <t>RTJ7E66</t>
@@ -1350,7 +1299,6 @@
           <t>FIORINO</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1387,8 +1335,6 @@
           <t>COTIA-EMBU-TABOAO,OSASCO-BARUERI-ALPHAVILLE,ZONA OESTE</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
           <t>PUX6D34</t>
@@ -1404,7 +1350,6 @@
           <t>FIORINO</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1441,8 +1386,6 @@
           <t>ZONA LESTE,ABCD,ZONA NORTE</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
           <t>NYA4J21</t>
@@ -1458,7 +1401,6 @@
           <t>FIORINO</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1498,7 +1440,6 @@
       <c r="I20" t="n">
         <v>11984344347</v>
       </c>
-      <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
           <t>FUP1D50</t>
@@ -1514,7 +1455,6 @@
           <t>FIORINO</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1574,13 +1514,11 @@
           <t>FIORINO</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
         <v>28438</v>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
           <t>Hugo Maçol Sousa (TESTE)</t>
@@ -1609,22 +1547,16 @@
           <t>ZONA NORTE,ZONA SUL,ZONA LESTE,ZONA OESTE,CENTRO,GUARULHOS,ABCD,OSASCO - BARUERI - SANTANA DE PARNAÍBA - ALPHAVILLE,COTIA - EMBU DAS ARTES - TABOÃO</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
           <t>11111111111</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
         <v>50190</v>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
           <t>Samuel Fugazza Neto</t>
@@ -1661,7 +1593,6 @@
           <t>sn@freshlog.com.br</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
           <t>42993322885</t>
@@ -1672,13 +1603,11 @@
           <t>FIORINO</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
         <v>50191</v>
       </c>
-      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
           <t>Iago Mendes</t>
@@ -1715,7 +1644,6 @@
           <t>im@freshlog.com.br</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
           <t>42640649884</t>
@@ -1726,7 +1654,6 @@
           <t>FIORINO</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1766,25 +1693,21 @@
       <c r="I25" t="n">
         <v>11995109716</v>
       </c>
-      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
           <t>EMU6742</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr">
         <is>
           <t>VAN_HR</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
         <v>50258</v>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
           <t>LALAMOVE (virtual)</t>
@@ -1795,7 +1718,6 @@
           <t>NAO</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="n">
         <v>99</v>
       </c>
@@ -1804,19 +1726,11 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
         <v>50219</v>
       </c>
-      <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
           <t>Diego Lopes</t>
@@ -1853,7 +1767,6 @@
           <t>dl@freshlog.com.br</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
           <t>38411793800</t>
@@ -1864,13 +1777,11 @@
           <t>VUC</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
         <v>46379</v>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
           <t>Patrícia Alexandre da Silva</t>
@@ -1899,22 +1810,16 @@
           <t>ZONA NORTE,ZONA SUL,ZONA LESTE,ZONA OESTE,CENTRO,GUARULHOS,ABCD,OSASCO-BARUERI-ALPHAVILLE,COTIA-EMBU-TABOAO</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr">
         <is>
           <t>VAN_HR</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
         <v>31861</v>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
           <t>Marlon Augusto Ribeiro Pumes</t>
@@ -1943,26 +1848,21 @@
           <t>ZONA SUL,ZONA NORTE,ZONA OESTE,ZONA LESTE</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr">
         <is>
           <t>RMZ1B04</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr">
         <is>
           <t>FIORINO</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
         <v>50826</v>
       </c>
-      <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
           <t>Maisa de Souza Leroz Silva</t>
@@ -1991,20 +1891,67 @@
           <t>ZONA SUL,ZONA NORTE,ZONA OESTE,ZONA LESTE</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
           <t>GDI5A39</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr">
         <is>
           <t>FIORINO</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>51410</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Rafael de Morais Coelho</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>SEGUNDA,TERCA,QUARTA,QUINTA,SEXTA</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>ZONA NORTE,ZONA SUL,ZONA LESTE,ZONA OESTE</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>5511988264183</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>RFK1H77</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>31880016818</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>FIORINO</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>